<commit_message>
Enhance Excel and Power BI dashboards
</commit_message>
<xml_diff>
--- a/dashboards/GrowthOps_OS_Excel_Dashboard.xlsx
+++ b/dashboards/GrowthOps_OS_Excel_Dashboard.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R109d235133d54f10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="2" r:id="R4bb6b630ff9a4c27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaigns" sheetId="3" r:id="R478f8a2b0cf3470a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel" sheetId="4" r:id="R0593ec3c82574c55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="5" r:id="Rc3e94e61ebc441f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="6" r:id="Raec43166df8040b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="7" r:id="R5b0bbdbef8ed481f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration" sheetId="8" r:id="Rd6975b57ddf04435"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Renewals" sheetId="9" r:id="R9c52b30adfc943f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue" sheetId="10" r:id="R5337664b449c4fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="11" r:id="Rb173218f33f24eee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1c3dc305d52b46e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis" sheetId="2" r:id="R9adc35e6d4224ecb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily" sheetId="3" r:id="Rab77d8ad83e34c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaigns" sheetId="4" r:id="Rccc1d9e6ca454fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel" sheetId="5" r:id="R1657f5cf3c934b4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="6" r:id="R51fb04489bab46c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="7" r:id="Raa9a2353bd3a4ea7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="8" r:id="Rf1fb5749902c448a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration" sheetId="9" r:id="Rfed0b615a5e546f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Renewals" sheetId="10" r:id="R650b8cb39129420c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue" sheetId="11" r:id="Rc5585156aa71435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="12" r:id="Ra6bcf2c25e8943a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,15 +24,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
     <x:numFmt numFmtId="203" formatCode="&quot;$&quot;#,##0"/>
     <x:numFmt numFmtId="204" formatCode="&quot;$&quot;#,##0.00"/>
     <x:numFmt numFmtId="205" formatCode="0.00&quot;x&quot;"/>
+    <x:numFmt numFmtId="206" formatCode="+0.0%;-0.0%;0.0%"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -67,12 +69,18 @@
     </x:font>
     <x:font>
       <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF173A5C"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
       <x:sz val="14"/>
       <x:color rgb="FF173A5C"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -89,6 +97,11 @@
         <x:fgColor rgb="FFEAF3F3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCECF8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -96,7 +109,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -114,7 +127,12 @@
     <x:xf numFmtId="203" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="204" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="205" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -401,6 +419,171 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/drawings/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr>
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:rPr>
+              <a:t>Weekly net cash and spend (USD)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr>
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Net cash (USD)</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Analysis'!$P$5:$P$19</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Analysis'!$Q$5:$Q$19</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Spend (USD)</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Analysis'!$P$5:$P$19</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Analysis'!$R$5:$R$19</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:smooth val="0"/>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
@@ -427,7 +610,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd3e05e912d784c88"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R35202fa14e78484f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -457,7 +640,42 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f9332fe0d7049ca"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7ee1f0677be040b6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2ee2106fd46546f5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1273,7 +1491,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="4" t="str">
-        <x:v>Due within seven days</x:v>
+        <x:v>Upcoming renewals (medium risk)</x:v>
       </x:c>
       <x:c r="B25" s="4" t="n">
         <x:f>COUNTIFS(Renewals!F2:F16,"medium")</x:f>
@@ -1480,7 +1698,9 @@
       <x:c r="O34" s="4"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="4"/>
+      <x:c r="A35" s="4" t="str">
+        <x:v>Use Analysis to change the reporting period and compare it with the prior period.</x:v>
+      </x:c>
       <x:c r="B35" s="4"/>
       <x:c r="C35" s="4"/>
       <x:c r="D35" s="4"/>
@@ -1566,11 +1786,348 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cfc27c6292d4777"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5638c1d3f1c74d2b"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="27" customHeight="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>subscription_id</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="str">
+        <x:v>customer_id</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="str">
+        <x:v>plan_id</x:v>
+      </x:c>
+      <x:c r="D1" s="2" t="str">
+        <x:v>due_date</x:v>
+      </x:c>
+      <x:c r="E1" s="2" t="str">
+        <x:v>failed_attempts</x:v>
+      </x:c>
+      <x:c r="F1" s="2" t="str">
+        <x:v>risk_level</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="4" t="str">
+        <x:v>sub-00176</x:v>
+      </x:c>
+      <x:c r="B2" s="4" t="str">
+        <x:v>c-00176</x:v>
+      </x:c>
+      <x:c r="C2" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D2" s="5" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="E2" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F2" s="4" t="str">
+        <x:v>high</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="4" t="str">
+        <x:v>sub-00000</x:v>
+      </x:c>
+      <x:c r="B3" s="4" t="str">
+        <x:v>c-00000</x:v>
+      </x:c>
+      <x:c r="C3" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D3" s="5" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="E3" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F3" s="4" t="str">
+        <x:v>high</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="4" t="str">
+        <x:v>sub-00064</x:v>
+      </x:c>
+      <x:c r="B4" s="4" t="str">
+        <x:v>c-00064</x:v>
+      </x:c>
+      <x:c r="C4" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="n">
+        <x:v>46292</x:v>
+      </x:c>
+      <x:c r="E4" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" s="4" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="4" t="str">
+        <x:v>sub-00208</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="str">
+        <x:v>c-00208</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D5" s="5" t="n">
+        <x:v>46292</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="4" t="str">
+        <x:v>sub-00096</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="str">
+        <x:v>c-00096</x:v>
+      </x:c>
+      <x:c r="C6" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="4" t="str">
+        <x:v>sub-00048</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="str">
+        <x:v>c-00048</x:v>
+      </x:c>
+      <x:c r="C7" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D7" s="5" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+      <x:c r="E7" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>not_due</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="4" t="str">
+        <x:v>sub-00144</x:v>
+      </x:c>
+      <x:c r="B8" s="4" t="str">
+        <x:v>c-00144</x:v>
+      </x:c>
+      <x:c r="C8" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="n">
+        <x:v>46303</x:v>
+      </x:c>
+      <x:c r="E8" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>not_due</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>sub-00192</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>c-00192</x:v>
+      </x:c>
+      <x:c r="C9" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D9" s="5" t="n">
+        <x:v>46312</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>not_due</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>sub-00080</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="str">
+        <x:v>c-00080</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D10" s="5" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E10" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="str">
+        <x:v>not_due</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>sub-00224</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>c-00224</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D11" s="5" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>not_due</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="4" t="str">
+        <x:v>sub-00016</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>c-00016</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>not_due</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>sub-00112</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>c-00112</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D13" s="5" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>not_due</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="4" t="str">
+        <x:v>sub-00160</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>c-00160</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D14" s="5" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>not_due</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="4" t="str">
+        <x:v>sub-00032</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>c-00032</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D15" s="5" t="n">
+        <x:v>46326</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>not_due</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="4" t="str">
+        <x:v>sub-00128</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>c-00128</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>founder_community</x:v>
+      </x:c>
+      <x:c r="D16" s="5" t="n">
+        <x:v>46344</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>not_due</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1613,7 +2170,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1622,7 +2179,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="17" t="str">
+      <x:c r="A1" s="22" t="str">
         <x:v>Reconciliation checks</x:v>
       </x:c>
     </x:row>
@@ -1672,6 +2229,1060 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF087F78"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="3" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="8" t="str">
+        <x:v>Period analysis and operating thresholds</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+      <x:c r="I1" s="4"/>
+      <x:c r="J1" s="4"/>
+      <x:c r="K1" s="4"/>
+      <x:c r="L1" s="4"/>
+      <x:c r="M1" s="4"/>
+      <x:c r="N1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="9" t="str">
+        <x:v>Edit the blue dates to compare an inclusive reporting window with the equally long prior window.</x:v>
+      </x:c>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+      <x:c r="D2" s="4"/>
+      <x:c r="E2" s="4"/>
+      <x:c r="F2" s="4"/>
+      <x:c r="G2" s="4"/>
+      <x:c r="H2" s="4"/>
+      <x:c r="I2" s="4"/>
+      <x:c r="J2" s="4"/>
+      <x:c r="K2" s="4"/>
+      <x:c r="L2" s="4"/>
+      <x:c r="M2" s="4"/>
+      <x:c r="N2" s="4"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="4"/>
+      <x:c r="B3" s="4"/>
+      <x:c r="C3" s="4"/>
+      <x:c r="D3" s="4"/>
+      <x:c r="E3" s="4"/>
+      <x:c r="F3" s="4"/>
+      <x:c r="G3" s="4"/>
+      <x:c r="H3" s="4"/>
+      <x:c r="I3" s="4"/>
+      <x:c r="J3" s="4"/>
+      <x:c r="K3" s="4"/>
+      <x:c r="L3" s="4"/>
+      <x:c r="M3" s="4"/>
+      <x:c r="N3" s="4"/>
+    </x:row>
+    <x:row r="4" ht="25" customHeight="1">
+      <x:c r="A4" s="4" t="str">
+        <x:v>Start date</x:v>
+      </x:c>
+      <x:c r="B4" s="18" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="C4" s="4"/>
+      <x:c r="D4" s="4"/>
+      <x:c r="E4" s="4"/>
+      <x:c r="F4" s="4"/>
+      <x:c r="G4" s="4"/>
+      <x:c r="H4" s="4"/>
+      <x:c r="I4" s="4"/>
+      <x:c r="J4" s="4"/>
+      <x:c r="K4" s="4"/>
+      <x:c r="L4" s="4"/>
+      <x:c r="M4" s="4"/>
+      <x:c r="N4" s="4"/>
+      <x:c r="P4" s="2" t="str">
+        <x:v>Week starting</x:v>
+      </x:c>
+      <x:c r="Q4" s="2" t="str">
+        <x:v>Net cash (USD)</x:v>
+      </x:c>
+      <x:c r="R4" s="2" t="str">
+        <x:v>Spend (USD)</x:v>
+      </x:c>
+      <x:c r="S4" s="2" t="str">
+        <x:v>Week start date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="25" customHeight="1">
+      <x:c r="A5" s="4" t="str">
+        <x:v>End date</x:v>
+      </x:c>
+      <x:c r="B5" s="18" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="C5" s="4"/>
+      <x:c r="D5" s="4"/>
+      <x:c r="E5" s="4"/>
+      <x:c r="F5" s="4"/>
+      <x:c r="G5" s="4"/>
+      <x:c r="H5" s="4"/>
+      <x:c r="I5" s="4"/>
+      <x:c r="J5" s="4"/>
+      <x:c r="K5" s="4"/>
+      <x:c r="L5" s="4"/>
+      <x:c r="M5" s="4"/>
+      <x:c r="N5" s="4"/>
+      <x:c r="P5" t="str">
+        <x:v>Jun 8</x:v>
+      </x:c>
+      <x:c r="Q5" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S5,Daily!A2:A99,"&lt;"&amp;S5+7)/100</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R5" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S5,Daily!A2:A99,"&lt;"&amp;S5+7)/100</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S5" s="20" t="n">
+        <x:v>46181</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="4" t="str">
+        <x:v>Days in window</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="n">
+        <x:f>B5-B4+1</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C6" s="4"/>
+      <x:c r="D6" s="4"/>
+      <x:c r="E6" s="4"/>
+      <x:c r="F6" s="4"/>
+      <x:c r="G6" s="4"/>
+      <x:c r="H6" s="4"/>
+      <x:c r="I6" s="4"/>
+      <x:c r="J6" s="4"/>
+      <x:c r="K6" s="4"/>
+      <x:c r="L6" s="4"/>
+      <x:c r="M6" s="4"/>
+      <x:c r="N6" s="4"/>
+      <x:c r="P6" t="str">
+        <x:v>Jun 15</x:v>
+      </x:c>
+      <x:c r="Q6" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S6,Daily!A2:A99,"&lt;"&amp;S6+7)/100</x:f>
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="R6" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S6,Daily!A2:A99,"&lt;"&amp;S6+7)/100</x:f>
+        <x:v>990.82</x:v>
+      </x:c>
+      <x:c r="S6" s="20" t="n">
+        <x:v>46188</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="4"/>
+      <x:c r="B7" s="4"/>
+      <x:c r="C7" s="4"/>
+      <x:c r="D7" s="4"/>
+      <x:c r="E7" s="4"/>
+      <x:c r="F7" s="4"/>
+      <x:c r="G7" s="4"/>
+      <x:c r="H7" s="4"/>
+      <x:c r="I7" s="4"/>
+      <x:c r="J7" s="4"/>
+      <x:c r="K7" s="4"/>
+      <x:c r="L7" s="4"/>
+      <x:c r="M7" s="4"/>
+      <x:c r="N7" s="4"/>
+      <x:c r="P7" t="str">
+        <x:v>Jun 22</x:v>
+      </x:c>
+      <x:c r="Q7" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S7,Daily!A2:A99,"&lt;"&amp;S7+7)/100</x:f>
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="R7" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S7,Daily!A2:A99,"&lt;"&amp;S7+7)/100</x:f>
+        <x:v>1104.52</x:v>
+      </x:c>
+      <x:c r="S7" s="20" t="n">
+        <x:v>46195</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="2" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="str">
+        <x:v>Selected window</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="str">
+        <x:v>Prior window</x:v>
+      </x:c>
+      <x:c r="D8" s="2" t="str">
+        <x:v>Change</x:v>
+      </x:c>
+      <x:c r="E8" s="4"/>
+      <x:c r="F8" s="4"/>
+      <x:c r="G8" s="4"/>
+      <x:c r="H8" s="4"/>
+      <x:c r="I8" s="4"/>
+      <x:c r="J8" s="4"/>
+      <x:c r="K8" s="4"/>
+      <x:c r="L8" s="4"/>
+      <x:c r="M8" s="4"/>
+      <x:c r="N8" s="4"/>
+      <x:c r="P8" t="str">
+        <x:v>Jun 29</x:v>
+      </x:c>
+      <x:c r="Q8" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S8,Daily!A2:A99,"&lt;"&amp;S8+7)/100</x:f>
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="R8" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S8,Daily!A2:A99,"&lt;"&amp;S8+7)/100</x:f>
+        <x:v>1005.27</x:v>
+      </x:c>
+      <x:c r="S8" s="20" t="n">
+        <x:v>46202</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="4" t="str">
+        <x:v>Spend (USD)</x:v>
+      </x:c>
+      <x:c r="B9" s="13" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;$B$4,Daily!A2:A99,"&lt;="&amp;$B$5)/100</x:f>
+        <x:v>3287.85</x:v>
+      </x:c>
+      <x:c r="C9" s="13" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;$B$4-$B$6,Daily!A2:A99,"&lt;="&amp;$B$4-1)/100</x:f>
+        <x:v>4466.54</x:v>
+      </x:c>
+      <x:c r="D9" s="19" t="n">
+        <x:f>IF(C9=0,"n.a.",B9/C9-1)</x:f>
+        <x:v>-0.26389330443699155</x:v>
+      </x:c>
+      <x:c r="E9" s="4"/>
+      <x:c r="F9" s="4"/>
+      <x:c r="G9" s="4"/>
+      <x:c r="H9" s="4"/>
+      <x:c r="I9" s="4"/>
+      <x:c r="J9" s="4"/>
+      <x:c r="K9" s="4"/>
+      <x:c r="L9" s="4"/>
+      <x:c r="M9" s="4"/>
+      <x:c r="N9" s="4"/>
+      <x:c r="P9" t="str">
+        <x:v>Jul 6</x:v>
+      </x:c>
+      <x:c r="Q9" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S9,Daily!A2:A99,"&lt;"&amp;S9+7)/100</x:f>
+        <x:v>-100</x:v>
+      </x:c>
+      <x:c r="R9" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S9,Daily!A2:A99,"&lt;"&amp;S9+7)/100</x:f>
+        <x:v>1056</x:v>
+      </x:c>
+      <x:c r="S9" s="20" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="4" t="str">
+        <x:v>Leads</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="n">
+        <x:f>SUMIFS(Daily!C2:C99,Daily!A2:A99,"&gt;="&amp;$B$4,Daily!A2:A99,"&lt;="&amp;$B$5)/1</x:f>
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="n">
+        <x:f>SUMIFS(Daily!C2:C99,Daily!A2:A99,"&gt;="&amp;$B$4-$B$6,Daily!A2:A99,"&lt;="&amp;$B$4-1)/1</x:f>
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="D10" s="19" t="n">
+        <x:f>IF(C10=0,"n.a.",B10/C10-1)</x:f>
+        <x:v>-0.7065217391304348</x:v>
+      </x:c>
+      <x:c r="E10" s="4"/>
+      <x:c r="F10" s="4"/>
+      <x:c r="G10" s="4"/>
+      <x:c r="H10" s="4"/>
+      <x:c r="I10" s="4"/>
+      <x:c r="J10" s="4"/>
+      <x:c r="K10" s="4"/>
+      <x:c r="L10" s="4"/>
+      <x:c r="M10" s="4"/>
+      <x:c r="N10" s="4"/>
+      <x:c r="P10" t="str">
+        <x:v>Jul 13</x:v>
+      </x:c>
+      <x:c r="Q10" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S10,Daily!A2:A99,"&lt;"&amp;S10+7)/100</x:f>
+        <x:v>2600</x:v>
+      </x:c>
+      <x:c r="R10" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S10,Daily!A2:A99,"&lt;"&amp;S10+7)/100</x:f>
+        <x:v>1054.89</x:v>
+      </x:c>
+      <x:c r="S10" s="20" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="4" t="str">
+        <x:v>MQLs</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="n">
+        <x:f>SUMIFS(Daily!D2:D99,Daily!A2:A99,"&gt;="&amp;$B$4,Daily!A2:A99,"&lt;="&amp;$B$5)/1</x:f>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="n">
+        <x:f>SUMIFS(Daily!D2:D99,Daily!A2:A99,"&gt;="&amp;$B$4-$B$6,Daily!A2:A99,"&lt;="&amp;$B$4-1)/1</x:f>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="D11" s="19" t="n">
+        <x:f>IF(C11=0,"n.a.",B11/C11-1)</x:f>
+        <x:v>-0.5714285714285714</x:v>
+      </x:c>
+      <x:c r="E11" s="4"/>
+      <x:c r="F11" s="4"/>
+      <x:c r="G11" s="4"/>
+      <x:c r="H11" s="4"/>
+      <x:c r="I11" s="4"/>
+      <x:c r="J11" s="4"/>
+      <x:c r="K11" s="4"/>
+      <x:c r="L11" s="4"/>
+      <x:c r="M11" s="4"/>
+      <x:c r="N11" s="4"/>
+      <x:c r="P11" t="str">
+        <x:v>Jul 20</x:v>
+      </x:c>
+      <x:c r="Q11" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S11,Daily!A2:A99,"&lt;"&amp;S11+7)/100</x:f>
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="R11" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S11,Daily!A2:A99,"&lt;"&amp;S11+7)/100</x:f>
+        <x:v>990.82</x:v>
+      </x:c>
+      <x:c r="S11" s="20" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="4" t="str">
+        <x:v>Calls booked</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="n">
+        <x:f>SUMIFS(Daily!E2:E99,Daily!A2:A99,"&gt;="&amp;$B$4,Daily!A2:A99,"&lt;="&amp;$B$5)/1</x:f>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="n">
+        <x:f>SUMIFS(Daily!E2:E99,Daily!A2:A99,"&gt;="&amp;$B$4-$B$6,Daily!A2:A99,"&lt;="&amp;$B$4-1)/1</x:f>
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="D12" s="19" t="n">
+        <x:f>IF(C12=0,"n.a.",B12/C12-1)</x:f>
+        <x:v>-0.5925925925925926</x:v>
+      </x:c>
+      <x:c r="E12" s="4"/>
+      <x:c r="F12" s="4"/>
+      <x:c r="G12" s="4"/>
+      <x:c r="H12" s="4"/>
+      <x:c r="I12" s="4"/>
+      <x:c r="J12" s="4"/>
+      <x:c r="K12" s="4"/>
+      <x:c r="L12" s="4"/>
+      <x:c r="M12" s="4"/>
+      <x:c r="N12" s="4"/>
+      <x:c r="P12" t="str">
+        <x:v>Jul 27</x:v>
+      </x:c>
+      <x:c r="Q12" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S12,Daily!A2:A99,"&lt;"&amp;S12+7)/100</x:f>
+        <x:v>2150</x:v>
+      </x:c>
+      <x:c r="R12" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S12,Daily!A2:A99,"&lt;"&amp;S12+7)/100</x:f>
+        <x:v>1104.44</x:v>
+      </x:c>
+      <x:c r="S12" s="20" t="n">
+        <x:v>46230</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="4" t="str">
+        <x:v>Booked value (USD)</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="n">
+        <x:f>SUMIFS(Daily!F2:F99,Daily!A2:A99,"&gt;="&amp;$B$4,Daily!A2:A99,"&lt;="&amp;$B$5)/100</x:f>
+        <x:v>3800</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="n">
+        <x:f>SUMIFS(Daily!F2:F99,Daily!A2:A99,"&gt;="&amp;$B$4-$B$6,Daily!A2:A99,"&lt;="&amp;$B$4-1)/100</x:f>
+        <x:v>10150</x:v>
+      </x:c>
+      <x:c r="D13" s="19" t="n">
+        <x:f>IF(C13=0,"n.a.",B13/C13-1)</x:f>
+        <x:v>-0.625615763546798</x:v>
+      </x:c>
+      <x:c r="E13" s="4"/>
+      <x:c r="F13" s="4"/>
+      <x:c r="G13" s="4"/>
+      <x:c r="H13" s="4"/>
+      <x:c r="I13" s="4"/>
+      <x:c r="J13" s="4"/>
+      <x:c r="K13" s="4"/>
+      <x:c r="L13" s="4"/>
+      <x:c r="M13" s="4"/>
+      <x:c r="N13" s="4"/>
+      <x:c r="P13" t="str">
+        <x:v>Aug 3</x:v>
+      </x:c>
+      <x:c r="Q13" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S13,Daily!A2:A99,"&lt;"&amp;S13+7)/100</x:f>
+        <x:v>1950</x:v>
+      </x:c>
+      <x:c r="R13" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S13,Daily!A2:A99,"&lt;"&amp;S13+7)/100</x:f>
+        <x:v>1005.13</x:v>
+      </x:c>
+      <x:c r="S13" s="20" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="4" t="str">
+        <x:v>Gross cash (USD)</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="n">
+        <x:f>SUMIFS(Daily!G2:G99,Daily!A2:A99,"&gt;="&amp;$B$4,Daily!A2:A99,"&lt;="&amp;$B$5)/100</x:f>
+        <x:v>3800</x:v>
+      </x:c>
+      <x:c r="C14" s="13" t="n">
+        <x:f>SUMIFS(Daily!G2:G99,Daily!A2:A99,"&gt;="&amp;$B$4-$B$6,Daily!A2:A99,"&lt;="&amp;$B$4-1)/100</x:f>
+        <x:v>10150</x:v>
+      </x:c>
+      <x:c r="D14" s="19" t="n">
+        <x:f>IF(C14=0,"n.a.",B14/C14-1)</x:f>
+        <x:v>-0.625615763546798</x:v>
+      </x:c>
+      <x:c r="E14" s="4"/>
+      <x:c r="F14" s="4"/>
+      <x:c r="G14" s="4"/>
+      <x:c r="H14" s="4"/>
+      <x:c r="I14" s="4"/>
+      <x:c r="J14" s="4"/>
+      <x:c r="K14" s="4"/>
+      <x:c r="L14" s="4"/>
+      <x:c r="M14" s="4"/>
+      <x:c r="N14" s="4"/>
+      <x:c r="P14" t="str">
+        <x:v>Aug 10</x:v>
+      </x:c>
+      <x:c r="Q14" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S14,Daily!A2:A99,"&lt;"&amp;S14+7)/100</x:f>
+        <x:v>2850</x:v>
+      </x:c>
+      <x:c r="R14" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S14,Daily!A2:A99,"&lt;"&amp;S14+7)/100</x:f>
+        <x:v>1055.86</x:v>
+      </x:c>
+      <x:c r="S14" s="20" t="n">
+        <x:v>46244</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="4" t="str">
+        <x:v>Refunds (USD)</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="n">
+        <x:f>SUMIFS(Daily!H2:H99,Daily!A2:A99,"&gt;="&amp;$B$4,Daily!A2:A99,"&lt;="&amp;$B$5)/100</x:f>
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="n">
+        <x:f>SUMIFS(Daily!H2:H99,Daily!A2:A99,"&gt;="&amp;$B$4-$B$6,Daily!A2:A99,"&lt;="&amp;$B$4-1)/100</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="D15" s="19" t="n">
+        <x:f>IF(C15=0,"n.a.",B15/C15-1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E15" s="4"/>
+      <x:c r="F15" s="4"/>
+      <x:c r="G15" s="4"/>
+      <x:c r="H15" s="4"/>
+      <x:c r="I15" s="4"/>
+      <x:c r="J15" s="4"/>
+      <x:c r="K15" s="4"/>
+      <x:c r="L15" s="4"/>
+      <x:c r="M15" s="4"/>
+      <x:c r="N15" s="4"/>
+      <x:c r="P15" t="str">
+        <x:v>Aug 17</x:v>
+      </x:c>
+      <x:c r="Q15" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S15,Daily!A2:A99,"&lt;"&amp;S15+7)/100</x:f>
+        <x:v>1300</x:v>
+      </x:c>
+      <x:c r="R15" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S15,Daily!A2:A99,"&lt;"&amp;S15+7)/100</x:f>
+        <x:v>1054.75</x:v>
+      </x:c>
+      <x:c r="S15" s="20" t="n">
+        <x:v>46251</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="4" t="str">
+        <x:v>Net cash (USD)</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;$B$4,Daily!A2:A99,"&lt;="&amp;$B$5)/100</x:f>
+        <x:v>3500</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;$B$4-$B$6,Daily!A2:A99,"&lt;="&amp;$B$4-1)/100</x:f>
+        <x:v>10050</x:v>
+      </x:c>
+      <x:c r="D16" s="19" t="n">
+        <x:f>IF(C16=0,"n.a.",B16/C16-1)</x:f>
+        <x:v>-0.6517412935323383</x:v>
+      </x:c>
+      <x:c r="E16" s="4"/>
+      <x:c r="F16" s="4"/>
+      <x:c r="G16" s="4"/>
+      <x:c r="H16" s="4"/>
+      <x:c r="I16" s="4"/>
+      <x:c r="J16" s="4"/>
+      <x:c r="K16" s="4"/>
+      <x:c r="L16" s="4"/>
+      <x:c r="M16" s="4"/>
+      <x:c r="N16" s="4"/>
+      <x:c r="P16" t="str">
+        <x:v>Aug 24</x:v>
+      </x:c>
+      <x:c r="Q16" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S16,Daily!A2:A99,"&lt;"&amp;S16+7)/100</x:f>
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="R16" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S16,Daily!A2:A99,"&lt;"&amp;S16+7)/100</x:f>
+        <x:v>990.68</x:v>
+      </x:c>
+      <x:c r="S16" s="20" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="4"/>
+      <x:c r="B17" s="4"/>
+      <x:c r="C17" s="4"/>
+      <x:c r="D17" s="4"/>
+      <x:c r="E17" s="4"/>
+      <x:c r="F17" s="4"/>
+      <x:c r="G17" s="4"/>
+      <x:c r="H17" s="4"/>
+      <x:c r="I17" s="4"/>
+      <x:c r="J17" s="4"/>
+      <x:c r="K17" s="4"/>
+      <x:c r="L17" s="4"/>
+      <x:c r="M17" s="4"/>
+      <x:c r="N17" s="4"/>
+      <x:c r="P17" t="str">
+        <x:v>Aug 31</x:v>
+      </x:c>
+      <x:c r="Q17" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S17,Daily!A2:A99,"&lt;"&amp;S17+7)/100</x:f>
+        <x:v>1300</x:v>
+      </x:c>
+      <x:c r="R17" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S17,Daily!A2:A99,"&lt;"&amp;S17+7)/100</x:f>
+        <x:v>1104.34</x:v>
+      </x:c>
+      <x:c r="S17" s="20" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2" t="str">
+        <x:v>Operating metric</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>Selected window</x:v>
+      </x:c>
+      <x:c r="C18" s="4"/>
+      <x:c r="D18" s="4"/>
+      <x:c r="E18" s="4"/>
+      <x:c r="F18" s="4"/>
+      <x:c r="G18" s="4"/>
+      <x:c r="H18" s="4"/>
+      <x:c r="I18" s="4"/>
+      <x:c r="J18" s="4"/>
+      <x:c r="K18" s="4"/>
+      <x:c r="L18" s="4"/>
+      <x:c r="M18" s="4"/>
+      <x:c r="N18" s="4"/>
+      <x:c r="P18" t="str">
+        <x:v>Sep 7</x:v>
+      </x:c>
+      <x:c r="Q18" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S18,Daily!A2:A99,"&lt;"&amp;S18+7)/100</x:f>
+        <x:v>1950</x:v>
+      </x:c>
+      <x:c r="R18" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S18,Daily!A2:A99,"&lt;"&amp;S18+7)/100</x:f>
+        <x:v>882.48</x:v>
+      </x:c>
+      <x:c r="S18" s="20" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="4" t="str">
+        <x:v>Lead to MQL</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="n">
+        <x:f>IF(B10=0,"n.a.",B11/B10)</x:f>
+        <x:v>0.5555555555555556</x:v>
+      </x:c>
+      <x:c r="C19" s="4"/>
+      <x:c r="D19" s="4"/>
+      <x:c r="E19" s="4"/>
+      <x:c r="F19" s="4"/>
+      <x:c r="G19" s="4"/>
+      <x:c r="H19" s="4"/>
+      <x:c r="I19" s="4"/>
+      <x:c r="J19" s="4"/>
+      <x:c r="K19" s="4"/>
+      <x:c r="L19" s="4"/>
+      <x:c r="M19" s="4"/>
+      <x:c r="N19" s="4"/>
+      <x:c r="P19" t="str">
+        <x:v>Sep 14</x:v>
+      </x:c>
+      <x:c r="Q19" s="21" t="n">
+        <x:f>SUMIFS(Daily!I2:I99,Daily!A2:A99,"&gt;="&amp;S19,Daily!A2:A99,"&lt;"&amp;S19+7)/100</x:f>
+        <x:v>-100</x:v>
+      </x:c>
+      <x:c r="R19" s="21" t="n">
+        <x:f>SUMIFS(Daily!B2:B99,Daily!A2:A99,"&gt;="&amp;S19,Daily!A2:A99,"&lt;"&amp;S19+7)/100</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S19" s="20" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="4" t="str">
+        <x:v>Paid cost per lead (USD)</x:v>
+      </x:c>
+      <x:c r="B20" s="15" t="n">
+        <x:f>IF(B10=0,"n.a.",B9/B10)</x:f>
+        <x:v>121.77222222222223</x:v>
+      </x:c>
+      <x:c r="C20" s="4"/>
+      <x:c r="D20" s="4"/>
+      <x:c r="E20" s="4"/>
+      <x:c r="F20" s="4"/>
+      <x:c r="G20" s="4"/>
+      <x:c r="H20" s="4"/>
+      <x:c r="I20" s="4"/>
+      <x:c r="J20" s="4"/>
+      <x:c r="K20" s="4"/>
+      <x:c r="L20" s="4"/>
+      <x:c r="M20" s="4"/>
+      <x:c r="N20" s="4"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="4" t="str">
+        <x:v>Cash to spend ratio</x:v>
+      </x:c>
+      <x:c r="B21" s="16" t="n">
+        <x:f>IF(B9=0,"n.a.",B16/B9)</x:f>
+        <x:v>1.0645254497620025</x:v>
+      </x:c>
+      <x:c r="C21" s="4"/>
+      <x:c r="D21" s="4"/>
+      <x:c r="E21" s="4"/>
+      <x:c r="F21" s="4"/>
+      <x:c r="G21" s="4"/>
+      <x:c r="H21" s="4"/>
+      <x:c r="I21" s="4"/>
+      <x:c r="J21" s="4"/>
+      <x:c r="K21" s="4"/>
+      <x:c r="L21" s="4"/>
+      <x:c r="M21" s="4"/>
+      <x:c r="N21" s="4"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="4"/>
+      <x:c r="B22" s="4"/>
+      <x:c r="C22" s="4"/>
+      <x:c r="D22" s="4"/>
+      <x:c r="E22" s="4"/>
+      <x:c r="F22" s="4"/>
+      <x:c r="G22" s="4"/>
+      <x:c r="H22" s="4"/>
+      <x:c r="I22" s="4"/>
+      <x:c r="J22" s="4"/>
+      <x:c r="K22" s="4"/>
+      <x:c r="L22" s="4"/>
+      <x:c r="M22" s="4"/>
+      <x:c r="N22" s="4"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2" t="str">
+        <x:v>Quality guardrail</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
+        <x:v>Target</x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E23" s="4"/>
+      <x:c r="F23" s="4"/>
+      <x:c r="G23" s="4"/>
+      <x:c r="H23" s="4"/>
+      <x:c r="I23" s="4"/>
+      <x:c r="J23" s="4"/>
+      <x:c r="K23" s="4"/>
+      <x:c r="L23" s="4"/>
+      <x:c r="M23" s="4"/>
+      <x:c r="N23" s="4"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="4" t="str">
+        <x:v>UTM completeness</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="n">
+        <x:f>Dashboard!B15</x:f>
+        <x:v>0.9343283582089552</x:v>
+      </x:c>
+      <x:c r="C24" s="7" t="n">
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="str">
+        <x:f>IF(B24&gt;=C24,"PASS","ACTION")</x:f>
+        <x:v>ACTION</x:v>
+      </x:c>
+      <x:c r="E24" s="4"/>
+      <x:c r="F24" s="4"/>
+      <x:c r="G24" s="4"/>
+      <x:c r="H24" s="4"/>
+      <x:c r="I24" s="4"/>
+      <x:c r="J24" s="4"/>
+      <x:c r="K24" s="4"/>
+      <x:c r="L24" s="4"/>
+      <x:c r="M24" s="4"/>
+      <x:c r="N24" s="4"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="4" t="str">
+        <x:v>Registry coverage</x:v>
+      </x:c>
+      <x:c r="B25" s="7" t="n">
+        <x:f>Dashboard!B16</x:f>
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="C25" s="7" t="n">
+        <x:v>0.98</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:f>IF(B25&gt;=C25,"PASS","ACTION")</x:f>
+        <x:v>ACTION</x:v>
+      </x:c>
+      <x:c r="E25" s="4"/>
+      <x:c r="F25" s="4"/>
+      <x:c r="G25" s="4"/>
+      <x:c r="H25" s="4"/>
+      <x:c r="I25" s="4"/>
+      <x:c r="J25" s="4"/>
+      <x:c r="K25" s="4"/>
+      <x:c r="L25" s="4"/>
+      <x:c r="M25" s="4"/>
+      <x:c r="N25" s="4"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="4" t="str">
+        <x:v>Owner coverage</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="n">
+        <x:f>Dashboard!B17</x:f>
+        <x:v>0.9375</x:v>
+      </x:c>
+      <x:c r="C26" s="7" t="n">
+        <x:v>0.99</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="str">
+        <x:f>IF(B26&gt;=C26,"PASS","ACTION")</x:f>
+        <x:v>ACTION</x:v>
+      </x:c>
+      <x:c r="E26" s="4"/>
+      <x:c r="F26" s="4"/>
+      <x:c r="G26" s="4"/>
+      <x:c r="H26" s="4"/>
+      <x:c r="I26" s="4"/>
+      <x:c r="J26" s="4"/>
+      <x:c r="K26" s="4"/>
+      <x:c r="L26" s="4"/>
+      <x:c r="M26" s="4"/>
+      <x:c r="N26" s="4"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="4"/>
+      <x:c r="B27" s="4"/>
+      <x:c r="C27" s="4"/>
+      <x:c r="D27" s="4"/>
+      <x:c r="E27" s="4"/>
+      <x:c r="F27" s="4"/>
+      <x:c r="G27" s="4"/>
+      <x:c r="H27" s="4"/>
+      <x:c r="I27" s="4"/>
+      <x:c r="J27" s="4"/>
+      <x:c r="K27" s="4"/>
+      <x:c r="L27" s="4"/>
+      <x:c r="M27" s="4"/>
+      <x:c r="N27" s="4"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="4" t="str">
+        <x:v>Reconciliation differences (cents)</x:v>
+      </x:c>
+      <x:c r="B28" s="4" t="n">
+        <x:f>SUM(ABS(Audit!B4),ABS(Audit!B5),ABS(Audit!B6))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C28" s="4"/>
+      <x:c r="D28" s="4"/>
+      <x:c r="E28" s="4"/>
+      <x:c r="F28" s="4"/>
+      <x:c r="G28" s="4"/>
+      <x:c r="H28" s="4"/>
+      <x:c r="I28" s="4"/>
+      <x:c r="J28" s="4"/>
+      <x:c r="K28" s="4"/>
+      <x:c r="L28" s="4"/>
+      <x:c r="M28" s="4"/>
+      <x:c r="N28" s="4"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="4"/>
+      <x:c r="B29" s="4"/>
+      <x:c r="C29" s="4"/>
+      <x:c r="D29" s="4"/>
+      <x:c r="E29" s="4"/>
+      <x:c r="F29" s="4"/>
+      <x:c r="G29" s="4"/>
+      <x:c r="H29" s="4"/>
+      <x:c r="I29" s="4"/>
+      <x:c r="J29" s="4"/>
+      <x:c r="K29" s="4"/>
+      <x:c r="L29" s="4"/>
+      <x:c r="M29" s="4"/>
+      <x:c r="N29" s="4"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="9" t="str">
+        <x:v>Scope: event-date daily cash; paid attribution and all-time revenue may differ by design.</x:v>
+      </x:c>
+      <x:c r="B30" s="4"/>
+      <x:c r="C30" s="4"/>
+      <x:c r="D30" s="4"/>
+      <x:c r="E30" s="4"/>
+      <x:c r="F30" s="4"/>
+      <x:c r="G30" s="4"/>
+      <x:c r="H30" s="4"/>
+      <x:c r="I30" s="4"/>
+      <x:c r="J30" s="4"/>
+      <x:c r="K30" s="4"/>
+      <x:c r="L30" s="4"/>
+      <x:c r="M30" s="4"/>
+      <x:c r="N30" s="4"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="9" t="str">
+        <x:v>Synthetic case data. Quality targets are operating defaults, not contractual SLAs.</x:v>
+      </x:c>
+      <x:c r="B31" s="4"/>
+      <x:c r="C31" s="4"/>
+      <x:c r="D31" s="4"/>
+      <x:c r="E31" s="4"/>
+      <x:c r="F31" s="4"/>
+      <x:c r="G31" s="4"/>
+      <x:c r="H31" s="4"/>
+      <x:c r="I31" s="4"/>
+      <x:c r="J31" s="4"/>
+      <x:c r="K31" s="4"/>
+      <x:c r="L31" s="4"/>
+      <x:c r="M31" s="4"/>
+      <x:c r="N31" s="4"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="4"/>
+      <x:c r="B32" s="4"/>
+      <x:c r="C32" s="4"/>
+      <x:c r="D32" s="4"/>
+      <x:c r="E32" s="4"/>
+      <x:c r="F32" s="4"/>
+      <x:c r="G32" s="4"/>
+      <x:c r="H32" s="4"/>
+      <x:c r="I32" s="4"/>
+      <x:c r="J32" s="4"/>
+      <x:c r="K32" s="4"/>
+      <x:c r="L32" s="4"/>
+      <x:c r="M32" s="4"/>
+      <x:c r="N32" s="4"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="4"/>
+      <x:c r="B33" s="4"/>
+      <x:c r="C33" s="4"/>
+      <x:c r="D33" s="4"/>
+      <x:c r="E33" s="4"/>
+      <x:c r="F33" s="4"/>
+      <x:c r="G33" s="4"/>
+      <x:c r="H33" s="4"/>
+      <x:c r="I33" s="4"/>
+      <x:c r="J33" s="4"/>
+      <x:c r="K33" s="4"/>
+      <x:c r="L33" s="4"/>
+      <x:c r="M33" s="4"/>
+      <x:c r="N33" s="4"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="4"/>
+      <x:c r="B34" s="4"/>
+      <x:c r="C34" s="4"/>
+      <x:c r="D34" s="4"/>
+      <x:c r="E34" s="4"/>
+      <x:c r="F34" s="4"/>
+      <x:c r="G34" s="4"/>
+      <x:c r="H34" s="4"/>
+      <x:c r="I34" s="4"/>
+      <x:c r="J34" s="4"/>
+      <x:c r="K34" s="4"/>
+      <x:c r="L34" s="4"/>
+      <x:c r="M34" s="4"/>
+      <x:c r="N34" s="4"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="4"/>
+      <x:c r="B35" s="4"/>
+      <x:c r="C35" s="4"/>
+      <x:c r="D35" s="4"/>
+      <x:c r="E35" s="4"/>
+      <x:c r="F35" s="4"/>
+      <x:c r="G35" s="4"/>
+      <x:c r="H35" s="4"/>
+      <x:c r="I35" s="4"/>
+      <x:c r="J35" s="4"/>
+      <x:c r="K35" s="4"/>
+      <x:c r="L35" s="4"/>
+      <x:c r="M35" s="4"/>
+      <x:c r="N35" s="4"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="4"/>
+      <x:c r="B36" s="4"/>
+      <x:c r="C36" s="4"/>
+      <x:c r="D36" s="4"/>
+      <x:c r="E36" s="4"/>
+      <x:c r="F36" s="4"/>
+      <x:c r="G36" s="4"/>
+      <x:c r="H36" s="4"/>
+      <x:c r="I36" s="4"/>
+      <x:c r="J36" s="4"/>
+      <x:c r="K36" s="4"/>
+      <x:c r="L36" s="4"/>
+      <x:c r="M36" s="4"/>
+      <x:c r="N36" s="4"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="4"/>
+      <x:c r="B37" s="4"/>
+      <x:c r="C37" s="4"/>
+      <x:c r="D37" s="4"/>
+      <x:c r="E37" s="4"/>
+      <x:c r="F37" s="4"/>
+      <x:c r="G37" s="4"/>
+      <x:c r="H37" s="4"/>
+      <x:c r="I37" s="4"/>
+      <x:c r="J37" s="4"/>
+      <x:c r="K37" s="4"/>
+      <x:c r="L37" s="4"/>
+      <x:c r="M37" s="4"/>
+      <x:c r="N37" s="4"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="4"/>
+      <x:c r="B38" s="4"/>
+      <x:c r="C38" s="4"/>
+      <x:c r="D38" s="4"/>
+      <x:c r="E38" s="4"/>
+      <x:c r="F38" s="4"/>
+      <x:c r="G38" s="4"/>
+      <x:c r="H38" s="4"/>
+      <x:c r="I38" s="4"/>
+      <x:c r="J38" s="4"/>
+      <x:c r="K38" s="4"/>
+      <x:c r="L38" s="4"/>
+      <x:c r="M38" s="4"/>
+      <x:c r="N38" s="4"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="4"/>
+      <x:c r="B39" s="4"/>
+      <x:c r="C39" s="4"/>
+      <x:c r="D39" s="4"/>
+      <x:c r="E39" s="4"/>
+      <x:c r="F39" s="4"/>
+      <x:c r="G39" s="4"/>
+      <x:c r="H39" s="4"/>
+      <x:c r="I39" s="4"/>
+      <x:c r="J39" s="4"/>
+      <x:c r="K39" s="4"/>
+      <x:c r="L39" s="4"/>
+      <x:c r="M39" s="4"/>
+      <x:c r="N39" s="4"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5d4f1d29d29459f"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4562,7 +6173,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4741,7 +6352,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4894,7 +6505,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -5203,7 +6814,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -5340,7 +6951,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -5425,7 +7036,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -5487,341 +7098,4 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="27" customHeight="1">
-      <x:c r="A1" s="2" t="str">
-        <x:v>subscription_id</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="str">
-        <x:v>customer_id</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="str">
-        <x:v>plan_id</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>due_date</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="str">
-        <x:v>failed_attempts</x:v>
-      </x:c>
-      <x:c r="F1" s="2" t="str">
-        <x:v>risk_level</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="4" t="str">
-        <x:v>sub-00176</x:v>
-      </x:c>
-      <x:c r="B2" s="4" t="str">
-        <x:v>c-00176</x:v>
-      </x:c>
-      <x:c r="C2" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D2" s="5" t="n">
-        <x:v>46281</x:v>
-      </x:c>
-      <x:c r="E2" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F2" s="4" t="str">
-        <x:v>high</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="4" t="str">
-        <x:v>sub-00000</x:v>
-      </x:c>
-      <x:c r="B3" s="4" t="str">
-        <x:v>c-00000</x:v>
-      </x:c>
-      <x:c r="C3" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D3" s="5" t="n">
-        <x:v>46282</x:v>
-      </x:c>
-      <x:c r="E3" s="4" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F3" s="4" t="str">
-        <x:v>high</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="22" customHeight="1">
-      <x:c r="A4" s="4" t="str">
-        <x:v>sub-00064</x:v>
-      </x:c>
-      <x:c r="B4" s="4" t="str">
-        <x:v>c-00064</x:v>
-      </x:c>
-      <x:c r="C4" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="n">
-        <x:v>46292</x:v>
-      </x:c>
-      <x:c r="E4" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F4" s="4" t="str">
-        <x:v>medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="22" customHeight="1">
-      <x:c r="A5" s="4" t="str">
-        <x:v>sub-00208</x:v>
-      </x:c>
-      <x:c r="B5" s="4" t="str">
-        <x:v>c-00208</x:v>
-      </x:c>
-      <x:c r="C5" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D5" s="5" t="n">
-        <x:v>46292</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="str">
-        <x:v>medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="22" customHeight="1">
-      <x:c r="A6" s="4" t="str">
-        <x:v>sub-00096</x:v>
-      </x:c>
-      <x:c r="B6" s="4" t="str">
-        <x:v>c-00096</x:v>
-      </x:c>
-      <x:c r="C6" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="n">
-        <x:v>46295</x:v>
-      </x:c>
-      <x:c r="E6" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F6" s="4" t="str">
-        <x:v>medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="22" customHeight="1">
-      <x:c r="A7" s="4" t="str">
-        <x:v>sub-00048</x:v>
-      </x:c>
-      <x:c r="B7" s="4" t="str">
-        <x:v>c-00048</x:v>
-      </x:c>
-      <x:c r="C7" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-      <x:c r="E7" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F7" s="4" t="str">
-        <x:v>not_due</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="22" customHeight="1">
-      <x:c r="A8" s="4" t="str">
-        <x:v>sub-00144</x:v>
-      </x:c>
-      <x:c r="B8" s="4" t="str">
-        <x:v>c-00144</x:v>
-      </x:c>
-      <x:c r="C8" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="n">
-        <x:v>46303</x:v>
-      </x:c>
-      <x:c r="E8" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F8" s="4" t="str">
-        <x:v>not_due</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="22" customHeight="1">
-      <x:c r="A9" s="4" t="str">
-        <x:v>sub-00192</x:v>
-      </x:c>
-      <x:c r="B9" s="4" t="str">
-        <x:v>c-00192</x:v>
-      </x:c>
-      <x:c r="C9" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="n">
-        <x:v>46312</x:v>
-      </x:c>
-      <x:c r="E9" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F9" s="4" t="str">
-        <x:v>not_due</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="22" customHeight="1">
-      <x:c r="A10" s="4" t="str">
-        <x:v>sub-00080</x:v>
-      </x:c>
-      <x:c r="B10" s="4" t="str">
-        <x:v>c-00080</x:v>
-      </x:c>
-      <x:c r="C10" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="n">
-        <x:v>46314</x:v>
-      </x:c>
-      <x:c r="E10" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F10" s="4" t="str">
-        <x:v>not_due</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="22" customHeight="1">
-      <x:c r="A11" s="4" t="str">
-        <x:v>sub-00224</x:v>
-      </x:c>
-      <x:c r="B11" s="4" t="str">
-        <x:v>c-00224</x:v>
-      </x:c>
-      <x:c r="C11" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="n">
-        <x:v>46316</x:v>
-      </x:c>
-      <x:c r="E11" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F11" s="4" t="str">
-        <x:v>not_due</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="22" customHeight="1">
-      <x:c r="A12" s="4" t="str">
-        <x:v>sub-00016</x:v>
-      </x:c>
-      <x:c r="B12" s="4" t="str">
-        <x:v>c-00016</x:v>
-      </x:c>
-      <x:c r="C12" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="n">
-        <x:v>46323</x:v>
-      </x:c>
-      <x:c r="E12" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F12" s="4" t="str">
-        <x:v>not_due</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="22" customHeight="1">
-      <x:c r="A13" s="4" t="str">
-        <x:v>sub-00112</x:v>
-      </x:c>
-      <x:c r="B13" s="4" t="str">
-        <x:v>c-00112</x:v>
-      </x:c>
-      <x:c r="C13" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D13" s="5" t="n">
-        <x:v>46323</x:v>
-      </x:c>
-      <x:c r="E13" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F13" s="4" t="str">
-        <x:v>not_due</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="22" customHeight="1">
-      <x:c r="A14" s="4" t="str">
-        <x:v>sub-00160</x:v>
-      </x:c>
-      <x:c r="B14" s="4" t="str">
-        <x:v>c-00160</x:v>
-      </x:c>
-      <x:c r="C14" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="n">
-        <x:v>46323</x:v>
-      </x:c>
-      <x:c r="E14" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F14" s="4" t="str">
-        <x:v>not_due</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="22" customHeight="1">
-      <x:c r="A15" s="4" t="str">
-        <x:v>sub-00032</x:v>
-      </x:c>
-      <x:c r="B15" s="4" t="str">
-        <x:v>c-00032</x:v>
-      </x:c>
-      <x:c r="C15" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D15" s="5" t="n">
-        <x:v>46326</x:v>
-      </x:c>
-      <x:c r="E15" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F15" s="4" t="str">
-        <x:v>not_due</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="22" customHeight="1">
-      <x:c r="A16" s="4" t="str">
-        <x:v>sub-00128</x:v>
-      </x:c>
-      <x:c r="B16" s="4" t="str">
-        <x:v>c-00128</x:v>
-      </x:c>
-      <x:c r="C16" s="4" t="str">
-        <x:v>founder_community</x:v>
-      </x:c>
-      <x:c r="D16" s="5" t="n">
-        <x:v>46344</x:v>
-      </x:c>
-      <x:c r="E16" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F16" s="4" t="str">
-        <x:v>not_due</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>